<commit_message>
feat(purchase-orders): add high-value business logic and data integrity negative test scenarios
</commit_message>
<xml_diff>
--- a/swarajya-update/purchase-orders/test_data/Update-Purchase-Order.xlsx
+++ b/swarajya-update/purchase-orders/test_data/Update-Purchase-Order.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +42,14 @@
       <color rgb="00006100"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="009C0006"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,6 +72,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="009C0006"/>
         <bgColor rgb="009C0006"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+        <bgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -111,6 +123,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1564,7 +1582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2105,6 +2123,188 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>TC_PO_NEG_09</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>Verify application rejects duplicate PO Reference Number assignment matching an existing PO</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>User is on /purchaseOrder with at least 2 PO records</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>1. Retrieve reference number from row 2
+2. Open edit modal for row 1
+3. Change PO Reference No to match row 2 reference number
+4. Click Update
+5. Verify duplicate collision rejection</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Existing Ref No from another record</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>Update is rejected with conflict error notification preventing duplicate PO Reference collision</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="inlineStr">
+        <is>
+          <t>AUTO_TC_PO_NEG_09</t>
+        </is>
+      </c>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>Data uniqueness constraint test</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>TC_PO_NEG_10</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>Verify application validates financial calculation consistency when Total Amount does not equal Base Amount plus Tax Amount</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>PO edit form is open</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>1. Set Base Amount to 5000
+2. Set Tax Amount to 500
+3. Set Total Amount to 99999
+4. Click Update
+5. Verify calculation consistency enforcement</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Base: 5000, Tax: 500, Total: 99999</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>Application validates amount consistency and blocks saving contradictory totals</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="inlineStr">
+        <is>
+          <t>AUTO_TC_PO_NEG_10</t>
+        </is>
+      </c>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>Financial Calculation Defect: System permitted saving contradictory amounts (Base: 5000 + Tax: 500 != Total: 99999)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>TC_PO_NEG_11</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>Verify application restricts modifying critical financial amounts and details on CANCELLED Purchase Orders</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>PO record is in CANCELLED status</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>1. Open edit modal for a CANCELLED PO
+2. Attempt to modify Base Amount or Total Amount
+3. Click Update
+4. Verify lifecycle rule restricts altering cancelled order terms</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Status: CANCELLED, modified amounts</t>
+        </is>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Cancelled PO records are locked or reject modification of financial terms without status reactivation</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="H12" s="6" t="inlineStr">
+        <is>
+          <t>Automated</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>AUTO_TC_PO_NEG_11</t>
+        </is>
+      </c>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>Lifecycle State Defect: System permitted modifying amounts on a CANCELLED Purchase Order without reactivation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(purchase-orders): separate positive and negative flows with FormExecutor architecture and 3 test suites
</commit_message>
<xml_diff>
--- a/swarajya-update/purchase-orders/test_data/Update-Purchase-Order.xlsx
+++ b/swarajya-update/purchase-orders/test_data/Update-Purchase-Order.xlsx
@@ -107,7 +107,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -129,6 +129,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -623,7 +626,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Edit modal opens with pre-populated data</t>
+          <t>Execution Passed Successfully (2.86s)</t>
         </is>
       </c>
     </row>
@@ -682,7 +685,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Customer Name is disabled/read-only</t>
+          <t>Execution Passed Successfully (2.32s)</t>
         </is>
       </c>
     </row>
@@ -741,7 +744,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Calendar picker toggle and popup verified</t>
+          <t>Execution Passed Successfully (3.74s)</t>
         </is>
       </c>
     </row>
@@ -800,7 +803,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>All specified currencies present and selectable</t>
+          <t>Execution Passed Successfully (3.94s)</t>
         </is>
       </c>
     </row>
@@ -859,7 +862,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>All 4 lifecycle status options verified</t>
+          <t>Execution Passed Successfully (3.87s)</t>
         </is>
       </c>
     </row>
@@ -918,7 +921,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>File upload and View Current Document link verified</t>
+          <t>Execution Passed Successfully (3.49s)</t>
         </is>
       </c>
     </row>
@@ -977,7 +980,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Cancel button retraction verified</t>
+          <t>Execution Passed Successfully (2.35s)</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1039,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Green success snackbar verified</t>
+          <t>Execution Passed Successfully (2.40s)</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1097,7 @@
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>Search by Ref No verified</t>
+          <t>Execution Passed Successfully (3.17s)</t>
         </is>
       </c>
     </row>
@@ -1153,7 +1156,7 @@
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>Include Fully Used PO filter verified</t>
+          <t>Execution Passed Successfully (5.66s)</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1215,7 @@
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>Status transition to PARTIALLY_USED verified</t>
+          <t>Execution Passed Successfully (6.94s)</t>
         </is>
       </c>
     </row>
@@ -1271,7 +1274,7 @@
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>Status transition to CANCELLED verified</t>
+          <t>Execution Passed Successfully (6.36s)</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1334,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>FULLY_USED transition and filter interplay verified</t>
+          <t>Execution Passed Successfully (9.76s)</t>
         </is>
       </c>
     </row>
@@ -1390,7 +1393,7 @@
       </c>
       <c r="K15" s="3" t="inlineStr">
         <is>
-          <t>Currency update persistence verified</t>
+          <t>Execution Passed Successfully (6.66s)</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1452,7 @@
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>PO Reference modification and search sync verified</t>
+          <t>Execution Passed Successfully (7.46s)</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1511,7 @@
       </c>
       <c r="K17" s="3" t="inlineStr">
         <is>
-          <t>Amount fields update verified</t>
+          <t>Execution Passed Successfully (2.84s)</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1570,7 @@
       </c>
       <c r="K18" s="3" t="inlineStr">
         <is>
-          <t>Document replacement verified</t>
+          <t>Execution Passed Successfully (3.47s)</t>
         </is>
       </c>
     </row>
@@ -1710,7 +1713,7 @@
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>Mandatory PO Details validation snackbar verified</t>
+          <t>Execution Passed Successfully (3.22s)</t>
         </is>
       </c>
     </row>
@@ -1768,7 +1771,7 @@
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>Customer Name rejected modification verified</t>
+          <t>Execution Passed Successfully (2.39s)</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1829,7 @@
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Non-existent search handled gracefully</t>
+          <t>Execution Passed Successfully (3.36s)</t>
         </is>
       </c>
     </row>
@@ -1884,7 +1887,7 @@
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>File input extension restriction verified</t>
+          <t>Execution Passed Successfully (2.29s)</t>
         </is>
       </c>
     </row>
@@ -1943,7 +1946,7 @@
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>Cancel preserved original listing data</t>
+          <t>Execution Passed Successfully (2.93s)</t>
         </is>
       </c>
     </row>
@@ -2002,7 +2005,7 @@
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>Modal close icon dismissal verified</t>
+          <t>Execution Passed Successfully (2.54s)</t>
         </is>
       </c>
     </row>
@@ -2061,7 +2064,7 @@
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>Search clear grid restoration verified</t>
+          <t>Execution Passed Successfully (6.40s)</t>
         </is>
       </c>
     </row>
@@ -2119,7 +2122,7 @@
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>Mandatory indicators verified</t>
+          <t>Execution Passed Successfully (2.34s)</t>
         </is>
       </c>
     </row>
@@ -2168,9 +2171,9 @@
           <t>Automated</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J10" s="6" t="inlineStr">
@@ -2180,7 +2183,12 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Data uniqueness constraint test</t>
+          <t>tests\test_po_update_negative_flows.py:30: in test_negative_scenario
+    executor.execute_negative_case(case)
+po_update_pages\form_executor.py:631: in execute_negative_case
+    assert is_rejected, (
+           ^^^^^^^^^^^
+E   AssertionError: Data Int (4.98s)</t>
         </is>
       </c>
     </row>
@@ -2241,7 +2249,12 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>Financial Calculation Defect: System permitted saving contradictory amounts (Base: 5000 + Tax: 500 != Total: 99999)</t>
+          <t>tests\test_po_update_negative_flows.py:30: in test_negative_scenario
+    executor.execute_negative_case(case)
+po_update_pages\form_executor.py:658: in execute_negative_case
+    assert is_rejected, (
+           ^^^^^^^^^^^
+E   AssertionError: Financia (5.80s)</t>
         </is>
       </c>
     </row>
@@ -2301,7 +2314,12 @@
       </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
-          <t>Lifecycle State Defect: System permitted modifying amounts on a CANCELLED Purchase Order without reactivation</t>
+          <t>tests\test_po_update_negative_flows.py:30: in test_negative_scenario
+    executor.execute_negative_case(case)
+po_update_pages\form_executor.py:694: in execute_negative_case
+    assert is_blocked, (
+           ^^^^^^^^^^
+E   AssertionError: Lifecycle  (9.37s)</t>
         </is>
       </c>
     </row>

</xml_diff>